<commit_message>
Refine UI and daily puzzle experience
</commit_message>
<xml_diff>
--- a/puzzels/netto_puzzels_race.xlsx
+++ b/puzzels/netto_puzzels_race.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Puzzels" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Puzzel Race" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Overzicht" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Niet gebruikt" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Daily Archive" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Puzzels" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Puzzel Race" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overzicht" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Niet gebruikt" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Archive" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Puzzels'!$A$1:$N$201</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Puzzel Race'!$A$1:$N$89</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Overzicht'!$A$1:$B$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Niet gebruikt'!$A$1:$D$123</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Daily Archive'!$A$1:$P$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Daily Archive'!$A$1:$P$36</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21052,7 +21052,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P29"/>
+  <dimension ref="A1:P36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -21166,51 +21166,51 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>+</t>
+          <t>−</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>9</v>
+        <v>1815</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Dieren</t>
+          <t>Geschiedenis</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel spelers staan er per team op het veld bij honkbal?</t>
+          <t>In welk jaar vond de Slag bij Waterloo plaats?</t>
         </is>
       </c>
       <c r="G2" s="2" t="n">
-        <v>2900</v>
+        <v>19</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Geografie</t>
+          <t>Boeken en literatuur</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel afzonderlijke riffen omvat het Great Barrier Reef ongeveer?</t>
+          <t>Hoeveel hoofdstukken bevat The Hobbit?</t>
         </is>
       </c>
       <c r="J2" s="2" t="n">
-        <v>2909</v>
+        <v>1796</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Gebouwen en infrastructuur</t>
+          <t>Biologie &amp; gezondheid</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel treden heeft de Burj Khalifa in Dubai?</t>
+          <t>In welk jaar werd het eerste succesvolle vaccin ontwikkeld?</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>9 + 2900 = 2909</t>
+          <t>1815 − 19 = 1796</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -21219,11 +21219,11 @@
         </is>
       </c>
       <c r="O2" s="2" t="n">
-        <v>79.26000000000001</v>
+        <v>86.15000000000001</v>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>library-154</t>
+          <t>library-169</t>
         </is>
       </c>
     </row>
@@ -21238,51 +21238,51 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>+</t>
+          <t>×</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>255</v>
+        <v>20</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Records en vergelijkingen</t>
+          <t>Spellen en speelgoed</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Hoe lang was de langste vrouw ooit in centimeters?</t>
+          <t>Hoeveel damstenen krijgt iedere speler bij de start van een standaard damspel?</t>
         </is>
       </c>
       <c r="G3" s="2" t="n">
-        <v>979</v>
+        <v>29</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Geografie</t>
+          <t>Taal</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel meter hoog is Angel Falls ongeveer?</t>
+          <t>Hoeveel letters heeft het Turkse alfabet?</t>
         </is>
       </c>
       <c r="J3" s="2" t="n">
-        <v>1234</v>
+        <v>580</v>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Natuurkunde</t>
+          <t>Eten &amp; drinken</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel kilometer per uur is de geluidssnelheid op zeeniveau afgerond?</t>
+          <t>Hoeveel kilocalorieën bevat een Amerikaanse McDonald’s Big Mac?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>255 + 979 = 1234</t>
+          <t>20 × 29 = 580</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -21291,11 +21291,11 @@
         </is>
       </c>
       <c r="O3" s="2" t="n">
-        <v>84.91</v>
+        <v>69.64</v>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>library-152</t>
+          <t>library-168</t>
         </is>
       </c>
     </row>
@@ -21310,51 +21310,51 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>÷</t>
+          <t>−</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>2700</v>
+        <v>775</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Dieren</t>
+          <t>Gebouwen en infrastructuur</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel kilogram weegt de tong van een blauwe vinvis ongeveer?</t>
+          <t>Hoeveel kamers heeft Buckingham Palace?</t>
         </is>
       </c>
       <c r="G4" s="2" t="n">
-        <v>15</v>
+        <v>687</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Politiek &amp; recht</t>
+          <t>Sterrenkunde &amp; ruimte</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel rechters telt het Internationaal Gerechtshof?</t>
+          <t>Hoeveel dagen doet de planeet Mars erover om rond de zon te draaien?</t>
         </is>
       </c>
       <c r="J4" s="2" t="n">
-        <v>180</v>
+        <v>88</v>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Wiskunde</t>
+          <t>Gebouwen en infrastructuur</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel graden heeft een gestrekte hoek?</t>
+          <t>Hoeveel verdiepingen hebben de Petronas Twin Towers?</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>2700 ÷ 15 = 180</t>
+          <t>775 − 687 = 88</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -21363,11 +21363,11 @@
         </is>
       </c>
       <c r="O4" s="2" t="n">
-        <v>86.93000000000001</v>
+        <v>84.77</v>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>library-150</t>
+          <t>library-167</t>
         </is>
       </c>
     </row>
@@ -21382,51 +21382,51 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>×</t>
+          <t>+</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>15</v>
+        <v>203</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Dieren</t>
+          <t>Records en vergelijkingen</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel kilo weegt een koningspinguin?</t>
+          <t>Hoe lang duurde de langste voetbalwedstrijd ooit in minuten?</t>
         </is>
       </c>
       <c r="G5" s="2" t="n">
-        <v>200</v>
+        <v>1247</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Geografie</t>
+          <t>Records en vergelijkingen</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel landen heeft Coca-Cola als afzetmarkt ongeveer?</t>
+          <t>Hoe zwaar was de zwaarste pompoen ooit in kilogram?</t>
         </is>
       </c>
       <c r="J5" s="2" t="n">
-        <v>3000</v>
+        <v>1450</v>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Landbouw en industrie</t>
+          <t>Technologie</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel ton goud wordt wereldwijd jaarlijks gewonnen?</t>
+          <t>In welk jaar werd de eerste drukpers met losse letters in Europa gebruikt?</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>15 × 200 = 3000</t>
+          <t>203 + 1247 = 1450</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -21435,11 +21435,11 @@
         </is>
       </c>
       <c r="O5" s="2" t="n">
-        <v>83.84999999999999</v>
+        <v>85.68000000000001</v>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>library-142</t>
+          <t>library-164</t>
         </is>
       </c>
     </row>
@@ -21454,51 +21454,51 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>÷</t>
+          <t>+</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>1215</v>
+        <v>134</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Geschiedenis</t>
+          <t>Gebouwen en infrastructuur</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>In welk jaar werd de Magna Carta bezegeld?</t>
+          <t>Hoeveel zuilen heeft de Grote Zuilenzaal van de Tempel van Karnak ongeveer?</t>
         </is>
       </c>
       <c r="G6" s="2" t="n">
-        <v>243</v>
+        <v>1642</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Sterrenkunde &amp; ruimte</t>
+          <t>Geografie</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel aardse dagen duurt één volledige draai van Venus ongeveer?</t>
+          <t>Wat is de diepte van het diepste zoetwatermeer ter wereld (Baikalmeer in Rusland) in meters?</t>
         </is>
       </c>
       <c r="J6" s="2" t="n">
-        <v>5</v>
+        <v>1776</v>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Sport</t>
+          <t>Gebouwen en infrastructuur</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel punten heeft een try in rugby union?</t>
+          <t>Hoeveel treden heeft de trap van de CN Tower ongeveer?</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>1215 ÷ 243 = 5</t>
+          <t>134 + 1642 = 1776</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -21507,11 +21507,11 @@
         </is>
       </c>
       <c r="O6" s="2" t="n">
-        <v>80.5</v>
+        <v>85.95999999999999</v>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>library-138</t>
+          <t>library-162</t>
         </is>
       </c>
     </row>
@@ -21526,51 +21526,51 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>×</t>
+          <t>÷</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>10</v>
+        <v>1665</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Dieren</t>
+          <t>Geschiedenis</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel poten heeft een krab?</t>
+          <t>In welk jaar werd de eerste moderne volkstelling gehouden?</t>
         </is>
       </c>
       <c r="G7" s="2" t="n">
-        <v>170</v>
+        <v>9</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Wiskunde</t>
+          <t>Filosofie, psychologie en religie</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel diagonalen heeft een regelmatige twintighoek?</t>
+          <t>Hoeveel Muzen (dochters van Zeus) telt de Griekse mythologie?</t>
         </is>
       </c>
       <c r="J7" s="2" t="n">
-        <v>1700</v>
+        <v>185</v>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Dagelijks leven</t>
+          <t>Nederlands</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel filialen heeft Decathlon wereldwijd ongeveer?</t>
+          <t>Hoe hoog is de Euromast in Rotterdam?</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>10 × 170 = 1700</t>
+          <t>1665 ÷ 9 = 185</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -21579,11 +21579,11 @@
         </is>
       </c>
       <c r="O7" s="2" t="n">
-        <v>79.05</v>
+        <v>82.91</v>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>library-125</t>
+          <t>library-157</t>
         </is>
       </c>
     </row>
@@ -21598,51 +21598,51 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>÷</t>
+          <t>+</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>1065</v>
+        <v>15</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Nederlands</t>
+          <t>Biologie &amp; gezondheid</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel kilometer fietst een Nederlander gemiddeld per jaar?</t>
+          <t>Hoeveel duizend knipperbewegingen met je ogen maak je gemiddeld per dag?</t>
         </is>
       </c>
       <c r="G8" s="2" t="n">
-        <v>15</v>
+        <v>538</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Nederlands</t>
+          <t>Politiek &amp; recht</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel tramlijnen heeft Amsterdam?</t>
+          <t>Hoeveel kiesmannen telt het Amerikaanse Electoral College?</t>
         </is>
       </c>
       <c r="J8" s="2" t="n">
-        <v>71</v>
+        <v>553</v>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Milieu en duurzaamheid</t>
+          <t>Gebouwen en infrastructuur</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Welk percentage van het aardoppervlak bestaat uit oceanen en zeeën?</t>
+          <t>Hoeveel meter hoog is de CN Tower?</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>1065 ÷ 15 = 71</t>
+          <t>15 + 538 = 553</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -21651,11 +21651,11 @@
         </is>
       </c>
       <c r="O8" s="2" t="n">
-        <v>78.89</v>
+        <v>66.79000000000001</v>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>library-124</t>
+          <t>library-155</t>
         </is>
       </c>
     </row>
@@ -21670,51 +21670,51 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>÷</t>
+          <t>+</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>1995</v>
+        <v>9</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Sterrenkunde &amp; ruimte</t>
+          <t>Dieren</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>In welk jaar werd de eerste exoplaneet rond een zonachtige ster ontdekt?</t>
+          <t>Hoeveel spelers staan er per team op het veld bij honkbal?</t>
         </is>
       </c>
       <c r="G9" s="2" t="n">
-        <v>57</v>
+        <v>2900</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
+          <t>Geografie</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Hoeveel afzonderlijke riffen omvat het Great Barrier Reef ongeveer?</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>2909</v>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
           <t>Gebouwen en infrastructuur</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>Hoeveel liften heeft de Burj Khalifa?</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>Wiskunde</t>
-        </is>
-      </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel diagonalen heeft een regelmatige tienhoek?</t>
+          <t>Hoeveel treden heeft de Burj Khalifa in Dubai?</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>1995 ÷ 57 = 35</t>
+          <t>9 + 2900 = 2909</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -21723,11 +21723,11 @@
         </is>
       </c>
       <c r="O9" s="2" t="n">
-        <v>84.2</v>
+        <v>79.26000000000001</v>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>library-112</t>
+          <t>library-154</t>
         </is>
       </c>
     </row>
@@ -21742,51 +21742,51 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>×</t>
+          <t>+</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>7</v>
+        <v>255</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Milieu en duurzaamheid</t>
+          <t>Records en vergelijkingen</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel procent van het Great Barrier Reef bestaat uit koraalriffen?</t>
+          <t>Hoe lang was de langste vrouw ooit in centimeters?</t>
         </is>
       </c>
       <c r="G10" s="2" t="n">
-        <v>44</v>
+        <v>979</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Taal</t>
+          <t>Geografie</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel letters heeft het Thaise alfabet?</t>
+          <t>Hoeveel meter hoog is Angel Falls ongeveer?</t>
         </is>
       </c>
       <c r="J10" s="2" t="n">
-        <v>308</v>
+        <v>1234</v>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Vervoer</t>
+          <t>Natuurkunde</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel metrostations heeft de Parijse metro?</t>
+          <t>Hoeveel kilometer per uur is de geluidssnelheid op zeeniveau afgerond?</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>7 × 44 = 308</t>
+          <t>255 + 979 = 1234</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -21795,11 +21795,11 @@
         </is>
       </c>
       <c r="O10" s="2" t="n">
-        <v>64.45999999999999</v>
+        <v>84.91</v>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>library-110</t>
+          <t>library-152</t>
         </is>
       </c>
     </row>
@@ -21818,47 +21818,47 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>1860</v>
+        <v>2700</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Gebouwen en infrastructuur</t>
+          <t>Dieren</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel treden heeft het Empire State Building van straatniveau tot het observatiedek?</t>
+          <t>Hoeveel kilogram weegt de tong van een blauwe vinvis ongeveer?</t>
         </is>
       </c>
       <c r="G11" s="2" t="n">
-        <v>62</v>
+        <v>15</v>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Films en series</t>
+          <t>Politiek &amp; recht</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel afleveringen telt de serie Breaking Bad?</t>
+          <t>Hoeveel rechters telt het Internationaal Gerechtshof?</t>
         </is>
       </c>
       <c r="J11" s="2" t="n">
-        <v>30</v>
+        <v>180</v>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Dieren</t>
+          <t>Wiskunde</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel kilometer per uur zwemt een dolfijn gemiddeld?</t>
+          <t>Hoeveel graden heeft een gestrekte hoek?</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>1860 ÷ 62 = 30</t>
+          <t>2700 ÷ 15 = 180</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -21867,11 +21867,11 @@
         </is>
       </c>
       <c r="O11" s="2" t="n">
-        <v>83.59999999999999</v>
+        <v>86.93000000000001</v>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>library-109</t>
+          <t>library-150</t>
         </is>
       </c>
     </row>
@@ -21886,51 +21886,51 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>÷</t>
+          <t>×</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>1989</v>
+        <v>15</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Technologie</t>
+          <t>Dieren</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>In welk jaar werd de eerste Nintendo Game Boy uitgebracht?</t>
+          <t>Hoeveel kilo weegt een koningspinguin?</t>
         </is>
       </c>
       <c r="G12" s="2" t="n">
-        <v>39</v>
+        <v>200</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Taal</t>
+          <t>Geografie</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel letters heeft het Armeense alfabet?</t>
+          <t>Hoeveel landen heeft Coca-Cola als afzetmarkt ongeveer?</t>
         </is>
       </c>
       <c r="J12" s="2" t="n">
-        <v>51</v>
+        <v>3000</v>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Records en vergelijkingen</t>
+          <t>Landbouw en industrie</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Hoe lang waren de langste mouwen aan een kledingstuk ooit in meters?</t>
+          <t>Hoeveel ton goud wordt wereldwijd jaarlijks gewonnen?</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>1989 ÷ 39 = 51</t>
+          <t>15 × 200 = 3000</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -21939,11 +21939,11 @@
         </is>
       </c>
       <c r="O12" s="2" t="n">
-        <v>84.17</v>
+        <v>83.84999999999999</v>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>library-107</t>
+          <t>library-142</t>
         </is>
       </c>
     </row>
@@ -21962,47 +21962,47 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>336</v>
+        <v>1215</v>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Wiskunde</t>
+          <t>Geschiedenis</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel manieren kun je 3 renners op een podium van 8 deelnemers indelen?</t>
+          <t>In welk jaar werd de Magna Carta bezegeld?</t>
         </is>
       </c>
       <c r="G13" s="2" t="n">
-        <v>21</v>
+        <v>243</v>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
+          <t>Sterrenkunde &amp; ruimte</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Hoeveel aardse dagen duurt één volledige draai van Venus ongeveer?</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
           <t>Sport</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>Hoeveel etappes telt de Tour de France doorgaans?</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>Biologie &amp; gezondheid</t>
-        </is>
-      </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel chromosomen heeft een gewone ui Allium cepa in een lichaamscel?</t>
+          <t>Hoeveel punten heeft een try in rugby union?</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>336 ÷ 21 = 16</t>
+          <t>1215 ÷ 243 = 5</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
@@ -22011,11 +22011,11 @@
         </is>
       </c>
       <c r="O13" s="2" t="n">
-        <v>69.01000000000001</v>
+        <v>80.5</v>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>library-106</t>
+          <t>library-138</t>
         </is>
       </c>
     </row>
@@ -22030,51 +22030,51 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>÷</t>
+          <t>×</t>
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>1164</v>
+        <v>10</v>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Records en vergelijkingen</t>
+          <t>Dieren</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Hoe zwaar was de zwaarste hamburger ooit in kilogram?</t>
+          <t>Hoeveel poten heeft een krab?</t>
         </is>
       </c>
       <c r="G14" s="2" t="n">
-        <v>97</v>
+        <v>170</v>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Records en vergelijkingen</t>
+          <t>Wiskunde</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel procent van het lichaam was bedekt met tatoeages bij de meest getatoeëerde man?</t>
+          <t>Hoeveel diagonalen heeft een regelmatige twintighoek?</t>
         </is>
       </c>
       <c r="J14" s="2" t="n">
-        <v>12</v>
+        <v>1700</v>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Films en series</t>
+          <t>Dagelijks leven</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel afleveringen telt de iconische serie Fawlty Towers?</t>
+          <t>Hoeveel filialen heeft Decathlon wereldwijd ongeveer?</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>1164 ÷ 97 = 12</t>
+          <t>10 × 170 = 1700</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -22083,11 +22083,11 @@
         </is>
       </c>
       <c r="O14" s="2" t="n">
-        <v>79.70999999999999</v>
+        <v>79.05</v>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>library-101</t>
+          <t>library-125</t>
         </is>
       </c>
     </row>
@@ -22102,51 +22102,51 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>×</t>
+          <t>÷</t>
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>6</v>
+        <v>1065</v>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Vervoer</t>
+          <t>Nederlands</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel start- en landingsbanen heeft Schiphol?</t>
+          <t>Hoeveel kilometer fietst een Nederlander gemiddeld per jaar?</t>
         </is>
       </c>
       <c r="G15" s="2" t="n">
-        <v>61</v>
+        <v>15</v>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Biologie &amp; gezondheid</t>
+          <t>Nederlands</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel toetsen heeft een standaard MIDI-pianotoetsenbord met vijf octaven?</t>
+          <t>Hoeveel tramlijnen heeft Amsterdam?</t>
         </is>
       </c>
       <c r="J15" s="2" t="n">
-        <v>366</v>
+        <v>71</v>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>Biologie &amp; gezondheid</t>
+          <t>Milieu en duurzaamheid</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel dagen telt een schrikkeljaar?</t>
+          <t>Welk percentage van het aardoppervlak bestaat uit oceanen en zeeën?</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>6 × 61 = 366</t>
+          <t>1065 ÷ 15 = 71</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
@@ -22155,11 +22155,11 @@
         </is>
       </c>
       <c r="O15" s="2" t="n">
-        <v>66.02</v>
+        <v>78.89</v>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>library-098</t>
+          <t>library-124</t>
         </is>
       </c>
     </row>
@@ -22178,47 +22178,47 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>636</v>
+        <v>1995</v>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Geografie</t>
+          <t>Sterrenkunde &amp; ruimte</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel kilometer lang is het Baikalmeer ongeveer?</t>
+          <t>In welk jaar werd de eerste exoplaneet rond een zonachtige ster ontdekt?</t>
         </is>
       </c>
       <c r="G16" s="2" t="n">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Kunst en cultuur</t>
+          <t>Gebouwen en infrastructuur</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel centimeter breed is de Mona Lisa?</t>
+          <t>Hoeveel liften heeft de Burj Khalifa?</t>
         </is>
       </c>
       <c r="J16" s="2" t="n">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Filosofie, psychologie en religie</t>
+          <t>Wiskunde</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel hoofdgoden telt de Griekse mythologie op de berg Olympus (de Twaalf Olympiërs)?</t>
+          <t>Hoeveel diagonalen heeft een regelmatige tienhoek?</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>636 ÷ 53 = 12</t>
+          <t>1995 ÷ 57 = 35</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
@@ -22227,11 +22227,11 @@
         </is>
       </c>
       <c r="O16" s="2" t="n">
-        <v>74.5</v>
+        <v>84.2</v>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>library-097</t>
+          <t>library-112</t>
         </is>
       </c>
     </row>
@@ -22246,37 +22246,37 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>÷</t>
+          <t>×</t>
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>1892</v>
+        <v>7</v>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Technologie</t>
+          <t>Milieu en duurzaamheid</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>In welk jaar werd de eerste internationale telefonische verbinding gemaakt?</t>
+          <t>Hoeveel procent van het Great Barrier Reef bestaat uit koraalriffen?</t>
         </is>
       </c>
       <c r="G17" s="2" t="n">
-        <v>86</v>
+        <v>44</v>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Biologie &amp; gezondheid</t>
+          <t>Taal</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel miljard neuronen (zenuwcellen) bevat het menselijk brein naar schatting?</t>
+          <t>Hoeveel letters heeft het Thaise alfabet?</t>
         </is>
       </c>
       <c r="J17" s="2" t="n">
-        <v>22</v>
+        <v>308</v>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
@@ -22285,12 +22285,12 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel wielen heeft een Airbus A380?</t>
+          <t>Hoeveel metrostations heeft de Parijse metro?</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>1892 ÷ 86 = 22</t>
+          <t>7 × 44 = 308</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
@@ -22299,11 +22299,11 @@
         </is>
       </c>
       <c r="O17" s="2" t="n">
-        <v>83.78</v>
+        <v>64.45999999999999</v>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>library-094</t>
+          <t>library-110</t>
         </is>
       </c>
     </row>
@@ -22318,51 +22318,51 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>×</t>
+          <t>÷</t>
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>35</v>
+        <v>1860</v>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Eten &amp; drinken</t>
+          <t>Gebouwen en infrastructuur</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel gram suiker zit er in een blikje Coca-Cola van 330 ml?</t>
+          <t>Hoeveel treden heeft het Empire State Building van straatniveau tot het observatiedek?</t>
         </is>
       </c>
       <c r="G18" s="2" t="n">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Muziek</t>
+          <t>Films en series</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel witte toetsen heeft een concertpiano?</t>
+          <t>Hoeveel afleveringen telt de serie Breaking Bad?</t>
         </is>
       </c>
       <c r="J18" s="2" t="n">
-        <v>1820</v>
+        <v>30</v>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>Geografie</t>
+          <t>Dieren</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>In welk jaar werd Antarctica voor het eerst waargenomen door een expeditie?</t>
+          <t>Hoeveel kilometer per uur zwemt een dolfijn gemiddeld?</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>35 × 52 = 1820</t>
+          <t>1860 ÷ 62 = 30</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
@@ -22371,11 +22371,11 @@
         </is>
       </c>
       <c r="O18" s="2" t="n">
-        <v>79.41</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>library-093</t>
+          <t>library-109</t>
         </is>
       </c>
     </row>
@@ -22394,47 +22394,47 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>1300</v>
+        <v>1989</v>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Spellen en speelgoed</t>
+          <t>Technologie</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel LEGO-steentjes worden er wereldwijd per seconde gemaakt?</t>
+          <t>In welk jaar werd de eerste Nintendo Game Boy uitgebracht?</t>
         </is>
       </c>
       <c r="G19" s="2" t="n">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Biologie &amp; gezondheid</t>
+          <t>Taal</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel speelkaarten zitten er in een standaard kaartspel (zonder jokers)?</t>
+          <t>Hoeveel letters heeft het Armeense alfabet?</t>
         </is>
       </c>
       <c r="J19" s="2" t="n">
-        <v>25</v>
+        <v>51</v>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Sterrenkunde &amp; ruimte</t>
+          <t>Records en vergelijkingen</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel aardse uren duurt één volledige draai van Mars ongeveer?</t>
+          <t>Hoe lang waren de langste mouwen aan een kledingstuk ooit in meters?</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>1300 ÷ 52 = 25</t>
+          <t>1989 ÷ 39 = 51</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
@@ -22443,11 +22443,11 @@
         </is>
       </c>
       <c r="O19" s="2" t="n">
-        <v>80.54000000000001</v>
+        <v>84.17</v>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>library-092</t>
+          <t>library-107</t>
         </is>
       </c>
     </row>
@@ -22466,47 +22466,47 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>1975</v>
+        <v>336</v>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Technologie</t>
+          <t>Wiskunde</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>In welk jaar werd de eerste digitale camera ontwikkeld?</t>
+          <t>Hoeveel manieren kun je 3 renners op een podium van 8 deelnemers indelen?</t>
         </is>
       </c>
       <c r="G20" s="2" t="n">
-        <v>79</v>
+        <v>21</v>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Scheikunde</t>
+          <t>Sport</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel protonen heeft een neutraal atoom van goud?</t>
+          <t>Hoeveel etappes telt de Tour de France doorgaans?</t>
         </is>
       </c>
       <c r="J20" s="2" t="n">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>Eten &amp; drinken</t>
+          <t>Biologie &amp; gezondheid</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel gram eiwit bevat een Amerikaanse McDonald’s Big Mac?</t>
+          <t>Hoeveel chromosomen heeft een gewone ui Allium cepa in een lichaamscel?</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>1975 ÷ 79 = 25</t>
+          <t>336 ÷ 21 = 16</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
@@ -22515,11 +22515,11 @@
         </is>
       </c>
       <c r="O20" s="2" t="n">
-        <v>84.14</v>
+        <v>69.01000000000001</v>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>library-090</t>
+          <t>library-106</t>
         </is>
       </c>
     </row>
@@ -22534,51 +22534,51 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>×</t>
+          <t>÷</t>
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>25</v>
+        <v>1164</v>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Natuurkunde</t>
+          <t>Records en vergelijkingen</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel millimeter per jaar verschuiven de aardplaten gemiddeld?</t>
+          <t>Hoe zwaar was de zwaarste hamburger ooit in kilogram?</t>
         </is>
       </c>
       <c r="G21" s="2" t="n">
-        <v>56</v>
+        <v>97</v>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Geschiedenis</t>
+          <t>Records en vergelijkingen</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel mannen ondertekenden de Amerikaanse Onafhankelijkheidsverklaring?</t>
+          <t>Hoeveel procent van het lichaam was bedekt met tatoeages bij de meest getatoeëerde man?</t>
         </is>
       </c>
       <c r="J21" s="2" t="n">
-        <v>1400</v>
+        <v>12</v>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>Technologie</t>
+          <t>Films en series</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>Wat is de totale lengte van alle onderzeese internetkabels op aarde in duizend kilometer?</t>
+          <t>Hoeveel afleveringen telt de iconische serie Fawlty Towers?</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>25 × 56 = 1400</t>
+          <t>1164 ÷ 97 = 12</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr">
@@ -22587,11 +22587,11 @@
         </is>
       </c>
       <c r="O21" s="2" t="n">
-        <v>77.17</v>
+        <v>79.70999999999999</v>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>library-088</t>
+          <t>library-101</t>
         </is>
       </c>
     </row>
@@ -22610,47 +22610,47 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Taal</t>
+          <t>Vervoer</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel letters heeft het Hebreeuwse alfabet?</t>
+          <t>Hoeveel start- en landingsbanen heeft Schiphol?</t>
         </is>
       </c>
       <c r="G22" s="2" t="n">
-        <v>82</v>
+        <v>61</v>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Wetenschap</t>
+          <t>Biologie &amp; gezondheid</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Wat is de lengte van het Panamakanaal van de Atlantische naar de Stille Oceaan in km?</t>
+          <t>Hoeveel toetsen heeft een standaard MIDI-pianotoetsenbord met vijf octaven?</t>
         </is>
       </c>
       <c r="J22" s="2" t="n">
-        <v>1804</v>
+        <v>366</v>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Vervoer</t>
+          <t>Biologie &amp; gezondheid</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>In welk jaar werd de eerste stoomlocomotief gebouwd?</t>
+          <t>Hoeveel dagen telt een schrikkeljaar?</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>22 × 82 = 1804</t>
+          <t>6 × 61 = 366</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr">
@@ -22659,11 +22659,11 @@
         </is>
       </c>
       <c r="O22" s="2" t="n">
-        <v>79.37</v>
+        <v>66.02</v>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>library-087</t>
+          <t>library-098</t>
         </is>
       </c>
     </row>
@@ -22678,51 +22678,51 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>×</t>
+          <t>÷</t>
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>50</v>
+        <v>636</v>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Milieu en duurzaamheid</t>
+          <t>Geografie</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel procent van de bekende plant- en diersoorten leeft in tropische regenwouden?</t>
+          <t>Hoeveel kilometer lang is het Baikalmeer ongeveer?</t>
         </is>
       </c>
       <c r="G23" s="2" t="n">
-        <v>101</v>
+        <v>53</v>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Gebouwen en infrastructuur</t>
+          <t>Kunst en cultuur</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel verdiepingen heeft Taipei 101?</t>
+          <t>Hoeveel centimeter breed is de Mona Lisa?</t>
         </is>
       </c>
       <c r="J23" s="2" t="n">
-        <v>5050</v>
+        <v>12</v>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>Wiskunde</t>
+          <t>Filosofie, psychologie en religie</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel is de som van de getallen 1 tot en met 100?</t>
+          <t>Hoeveel hoofdgoden telt de Griekse mythologie op de berg Olympus (de Twaalf Olympiërs)?</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>50 × 101 = 5050</t>
+          <t>636 ÷ 53 = 12</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr">
@@ -22731,11 +22731,11 @@
         </is>
       </c>
       <c r="O23" s="2" t="n">
-        <v>88.2</v>
+        <v>74.5</v>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>library-083</t>
+          <t>library-097</t>
         </is>
       </c>
     </row>
@@ -22750,51 +22750,51 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>×</t>
+          <t>÷</t>
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>35</v>
+        <v>1892</v>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Muziek</t>
+          <t>Technologie</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel Grammy’s heeft Beyoncé volgens de stand na de Grammy Awards van 2025 gewonnen?</t>
+          <t>In welk jaar werd de eerste internationale telefonische verbinding gemaakt?</t>
         </is>
       </c>
       <c r="G24" s="2" t="n">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Landbouw en industrie</t>
+          <t>Biologie &amp; gezondheid</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>Welk percentage van het wereldwijde cement wordt geproduceerd in China?</t>
+          <t>Hoeveel miljard neuronen (zenuwcellen) bevat het menselijk brein naar schatting?</t>
         </is>
       </c>
       <c r="J24" s="2" t="n">
-        <v>1925</v>
+        <v>22</v>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>Technologie</t>
+          <t>Vervoer</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>In welk jaar werd de eerste televisie-uitzending verzorgd?</t>
+          <t>Hoeveel wielen heeft een Airbus A380?</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>35 × 55 = 1925</t>
+          <t>1892 ÷ 86 = 22</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr">
@@ -22803,11 +22803,11 @@
         </is>
       </c>
       <c r="O24" s="2" t="n">
-        <v>79.89</v>
+        <v>83.78</v>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>library-081</t>
+          <t>library-094</t>
         </is>
       </c>
     </row>
@@ -22826,47 +22826,47 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
+          <t>Eten &amp; drinken</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Hoeveel gram suiker zit er in een blikje Coca-Cola van 330 ml?</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
           <t>Muziek</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>Hoeveel halve tonen bevat een octaaf?</t>
-        </is>
-      </c>
-      <c r="G25" s="2" t="n">
-        <v>69</v>
-      </c>
-      <c r="H25" s="2" t="inlineStr">
-        <is>
-          <t>Milieu en duurzaamheid</t>
-        </is>
-      </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>Welk percentage van het zoete water zit vast in ijs en gletsjers?</t>
+          <t>Hoeveel witte toetsen heeft een concertpiano?</t>
         </is>
       </c>
       <c r="J25" s="2" t="n">
-        <v>828</v>
+        <v>1820</v>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>Gebouwen en infrastructuur</t>
+          <t>Geografie</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>Wat is de hoogte van de Burj Khalifa in Dubai in meters?</t>
+          <t>In welk jaar werd Antarctica voor het eerst waargenomen door een expeditie?</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>12 × 69 = 828</t>
+          <t>35 × 52 = 1820</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr">
@@ -22875,11 +22875,11 @@
         </is>
       </c>
       <c r="O25" s="2" t="n">
-        <v>72.78</v>
+        <v>79.41</v>
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>library-080</t>
+          <t>library-093</t>
         </is>
       </c>
     </row>
@@ -22894,37 +22894,37 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>×</t>
+          <t>÷</t>
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>20</v>
+        <v>1300</v>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Gebouwen en infrastructuur</t>
+          <t>Spellen en speelgoed</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel torens heeft het Kremlin in Moskou?</t>
+          <t>Hoeveel LEGO-steentjes worden er wereldwijd per seconde gemaakt?</t>
         </is>
       </c>
       <c r="G26" s="2" t="n">
-        <v>227</v>
+        <v>52</v>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Vervoer</t>
+          <t>Biologie &amp; gezondheid</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel meter hoog is de Golden Gate Bridge boven het water?</t>
+          <t>Hoeveel speelkaarten zitten er in een standaard kaartspel (zonder jokers)?</t>
         </is>
       </c>
       <c r="J26" s="2" t="n">
-        <v>4540</v>
+        <v>25</v>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
@@ -22933,12 +22933,12 @@
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>Wat is de geschatte leeftijd van de planeet Aarde in miljoenen jaren?</t>
+          <t>Hoeveel aardse uren duurt één volledige draai van Mars ongeveer?</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>20 × 227 = 4540</t>
+          <t>1300 ÷ 52 = 25</t>
         </is>
       </c>
       <c r="N26" s="2" t="inlineStr">
@@ -22947,11 +22947,11 @@
         </is>
       </c>
       <c r="O26" s="2" t="n">
-        <v>87.37</v>
+        <v>80.54000000000001</v>
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>library-078</t>
+          <t>library-092</t>
         </is>
       </c>
     </row>
@@ -22966,51 +22966,51 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>×</t>
+          <t>÷</t>
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>5</v>
+        <v>1975</v>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Geografie</t>
+          <t>Technologie</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel landen grenzen aan Zwitserland?</t>
+          <t>In welk jaar werd de eerste digitale camera ontwikkeld?</t>
         </is>
       </c>
       <c r="G27" s="2" t="n">
-        <v>163</v>
+        <v>79</v>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>Gebouwen en infrastructuur</t>
+          <t>Scheikunde</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel verdiepingen heeft de Burj Khalifa?</t>
+          <t>Hoeveel protonen heeft een neutraal atoom van goud?</t>
         </is>
       </c>
       <c r="J27" s="2" t="n">
-        <v>815</v>
+        <v>25</v>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>Records en vergelijkingen</t>
+          <t>Eten &amp; drinken</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>Hoe groot was het grootste permanente IMAX-scherm in vierkante meter?</t>
+          <t>Hoeveel gram eiwit bevat een Amerikaanse McDonald’s Big Mac?</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>5 × 163 = 815</t>
+          <t>1975 ÷ 79 = 25</t>
         </is>
       </c>
       <c r="N27" s="2" t="inlineStr">
@@ -23019,11 +23019,11 @@
         </is>
       </c>
       <c r="O27" s="2" t="n">
-        <v>73.05</v>
+        <v>84.14</v>
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>library-074</t>
+          <t>library-090</t>
         </is>
       </c>
     </row>
@@ -23042,20 +23042,20 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Milieu en duurzaamheid</t>
+          <t>Natuurkunde</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Welk percentage van het aardoppervlak bestaat uit land?</t>
+          <t>Hoeveel millimeter per jaar verschuiven de aardplaten gemiddeld?</t>
         </is>
       </c>
       <c r="G28" s="2" t="n">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
@@ -23064,25 +23064,25 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>Hoeveel dagen duurde de reis van de Mayflower naar Noord-Amerika?</t>
+          <t>Hoeveel mannen ondertekenden de Amerikaanse Onafhankelijkheidsverklaring?</t>
         </is>
       </c>
       <c r="J28" s="2" t="n">
-        <v>1914</v>
+        <v>1400</v>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>Vervoer</t>
+          <t>Technologie</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>In welk jaar vertrok de eerste commerciële passagiersvlucht?</t>
+          <t>Wat is de totale lengte van alle onderzeese internetkabels op aarde in duizend kilometer?</t>
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>29 × 66 = 1914</t>
+          <t>25 × 56 = 1400</t>
         </is>
       </c>
       <c r="N28" s="2" t="inlineStr">
@@ -23091,11 +23091,11 @@
         </is>
       </c>
       <c r="O28" s="2" t="n">
-        <v>79.84999999999999</v>
+        <v>77.17</v>
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>library-073</t>
+          <t>library-088</t>
         </is>
       </c>
     </row>
@@ -23114,65 +23114,569 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Taal</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Hoeveel letters heeft het Hebreeuwse alfabet?</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Wetenschap</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>Wat is de lengte van het Panamakanaal van de Atlantische naar de Stille Oceaan in km?</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="n">
+        <v>1804</v>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>Vervoer</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>In welk jaar werd de eerste stoomlocomotief gebouwd?</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>22 × 82 = 1804</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="O29" s="2" t="n">
+        <v>79.37</v>
+      </c>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>library-087</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>×</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Milieu en duurzaamheid</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Hoeveel procent van de bekende plant- en diersoorten leeft in tropische regenwouden?</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>101</v>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Gebouwen en infrastructuur</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Hoeveel verdiepingen heeft Taipei 101?</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="n">
+        <v>5050</v>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Wiskunde</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>Hoeveel is de som van de getallen 1 tot en met 100?</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>50 × 101 = 5050</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="n">
+        <v>88.2</v>
+      </c>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>library-083</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>×</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Muziek</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Hoeveel Grammy’s heeft Beyoncé volgens de stand na de Grammy Awards van 2025 gewonnen?</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Landbouw en industrie</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>Welk percentage van het wereldwijde cement wordt geproduceerd in China?</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="n">
+        <v>1925</v>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Technologie</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>In welk jaar werd de eerste televisie-uitzending verzorgd?</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>35 × 55 = 1925</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="O31" s="2" t="n">
+        <v>79.89</v>
+      </c>
+      <c r="P31" s="2" t="inlineStr">
+        <is>
+          <t>library-081</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>×</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Muziek</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Hoeveel halve tonen bevat een octaaf?</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Milieu en duurzaamheid</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Welk percentage van het zoete water zit vast in ijs en gletsjers?</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="n">
+        <v>828</v>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Gebouwen en infrastructuur</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>Wat is de hoogte van de Burj Khalifa in Dubai in meters?</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>12 × 69 = 828</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="O32" s="2" t="n">
+        <v>72.78</v>
+      </c>
+      <c r="P32" s="2" t="inlineStr">
+        <is>
+          <t>library-080</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>×</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Gebouwen en infrastructuur</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Hoeveel torens heeft het Kremlin in Moskou?</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>227</v>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Vervoer</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>Hoeveel meter hoog is de Golden Gate Bridge boven het water?</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="n">
+        <v>4540</v>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>Sterrenkunde &amp; ruimte</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>Wat is de geschatte leeftijd van de planeet Aarde in miljoenen jaren?</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>20 × 227 = 4540</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="O33" s="2" t="n">
+        <v>87.37</v>
+      </c>
+      <c r="P33" s="2" t="inlineStr">
+        <is>
+          <t>library-078</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>×</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Geografie</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Hoeveel landen grenzen aan Zwitserland?</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>163</v>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Gebouwen en infrastructuur</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>Hoeveel verdiepingen heeft de Burj Khalifa?</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="n">
+        <v>815</v>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>Records en vergelijkingen</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>Hoe groot was het grootste permanente IMAX-scherm in vierkante meter?</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>5 × 163 = 815</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="O34" s="2" t="n">
+        <v>73.05</v>
+      </c>
+      <c r="P34" s="2" t="inlineStr">
+        <is>
+          <t>library-074</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>×</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Milieu en duurzaamheid</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Welk percentage van het aardoppervlak bestaat uit land?</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Geschiedenis</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>Hoeveel dagen duurde de reis van de Mayflower naar Noord-Amerika?</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="n">
+        <v>1914</v>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>Vervoer</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>In welk jaar vertrok de eerste commerciële passagiersvlucht?</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>29 × 66 = 1914</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="O35" s="2" t="n">
+        <v>79.84999999999999</v>
+      </c>
+      <c r="P35" s="2" t="inlineStr">
+        <is>
+          <t>library-073</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>×</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>Taal</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>Hoeveel naamvallen heeft het Fins?</t>
         </is>
       </c>
-      <c r="G29" s="2" t="n">
+      <c r="G36" s="2" t="n">
         <v>98</v>
       </c>
-      <c r="H29" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t>Geografie</t>
         </is>
       </c>
-      <c r="I29" s="2" t="inlineStr">
+      <c r="I36" s="2" t="inlineStr">
         <is>
           <t>Hoeveel procent van Antarctica is met ijs bedekt?</t>
         </is>
       </c>
-      <c r="J29" s="2" t="n">
+      <c r="J36" s="2" t="n">
         <v>1470</v>
       </c>
-      <c r="K29" s="2" t="inlineStr">
+      <c r="K36" s="2" t="inlineStr">
         <is>
           <t>Geografie</t>
         </is>
       </c>
-      <c r="L29" s="2" t="inlineStr">
+      <c r="L36" s="2" t="inlineStr">
         <is>
           <t>Hoeveel meter diep is het Tanganyikameer op het diepste punt ongeveer?</t>
         </is>
       </c>
-      <c r="M29" s="2" t="inlineStr">
+      <c r="M36" s="2" t="inlineStr">
         <is>
           <t>15 × 98 = 1470</t>
         </is>
       </c>
-      <c r="N29" s="2" t="inlineStr">
+      <c r="N36" s="2" t="inlineStr">
         <is>
           <t>hard</t>
         </is>
       </c>
-      <c r="O29" s="2" t="n">
+      <c r="O36" s="2" t="n">
         <v>77.67</v>
       </c>
-      <c r="P29" s="2" t="inlineStr">
+      <c r="P36" s="2" t="inlineStr">
         <is>
           <t>library-072</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P29"/>
+  <autoFilter ref="A1:P36"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>